<commit_message>
Keep synthetic demo output out of data/normalized
The demo run wrote its synthetic rows to data/normalized/, where they could be
mistaken for real listings. Demo mode now writes only to its output folder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017BXrUCfQ5bzXFxVzCV3UDj
</commit_message>
<xml_diff>
--- a/docs/preview/PREVIEW_SYNTHETIC_Miraflores_Rental_Shortlist.xlsx
+++ b/docs/preview/PREVIEW_SYNTHETIC_Miraflores_Rental_Shortlist.xlsx
@@ -860,7 +860,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback) · Budget-compliant (rent ≤ USD 1,000), 1–2 bedrooms, inside Miraflores. Availability as checked at the QA timestamp; not guaranteed.</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback) · Budget-compliant (rent ≤ USD 1,000), 1–2 bedrooms, inside Miraflores. Availability as checked at the QA timestamp; not guaranteed.</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>
@@ -10659,7 +10659,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>
@@ -13249,7 +13249,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>
@@ -13857,7 +13857,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>
@@ -14817,7 +14817,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>
@@ -14872,7 +14872,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00. Listings collected: 41; unique after de-duplication: 40; budget-compliant matches: 26; stretch: 9; near misses: 1. External cost: USD 0.00.</t>
+          <t>Generated 2026-09-24T17:45:37-05:00. Listings collected: 41; unique after de-duplication: 40; budget-compliant matches: 26; stretch: 9; near misses: 1. External cost: USD 0.00.</t>
         </is>
       </c>
     </row>
@@ -14884,7 +14884,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>1 USD = S/ 3.385 · SYNTHETIC DEMO RATE (same value as documented fallback) · 2026-09-24T17:45:06-05:00. Used for every conversion. Values published by the listing are marked PUBLISHED; converted values CALCULATED. When a listing publishes both currencies, both are kept as published.</t>
+          <t>1 USD = S/ 3.385 · SYNTHETIC DEMO RATE (same value as documented fallback) · 2026-09-24T17:45:37-05:00. Used for every conversion. Values published by the listing are marked PUBLISHED; converted values CALCULATED. When a listing publishes both currencies, both are kept as published.</t>
         </is>
       </c>
     </row>
@@ -15064,7 +15064,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-24T17:45:06-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
+          <t>Generated 2026-09-24T17:45:37-05:00 · FX 1 USD = S/ 3.385 (fallback)</t>
         </is>
       </c>
     </row>

</xml_diff>